<commit_message>
Update INARA 2026-09-30 10:24:45
</commit_message>
<xml_diff>
--- a/summary_odp_black_special_value_hq.xlsx
+++ b/summary_odp_black_special_value_hq.xlsx
@@ -531,10 +531,10 @@
         <v>100</v>
       </c>
       <c r="F2">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="G2">
-        <v>4.43</v>
+        <v>4.45</v>
       </c>
       <c r="H2">
         <v>27</v>
@@ -663,10 +663,10 @@
         <v>100</v>
       </c>
       <c r="F5">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G5">
-        <v>1.97</v>
+        <v>2</v>
       </c>
       <c r="H5">
         <v>24</v>
@@ -839,10 +839,10 @@
         <v>100</v>
       </c>
       <c r="F9">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G9">
-        <v>1.97</v>
+        <v>2</v>
       </c>
       <c r="H9">
         <v>24</v>
@@ -1015,10 +1015,10 @@
         <v>100</v>
       </c>
       <c r="F13">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G13">
-        <v>1.53</v>
+        <v>1.58</v>
       </c>
       <c r="H13">
         <v>16</v>

</xml_diff>